<commit_message>
Update FSEOF terminology and refresh 2,3-BDO FSEOF results
</commit_message>
<xml_diff>
--- a/FSEOF_results_v2_564.xlsx
+++ b/FSEOF_results_v2_564.xlsx
@@ -7940,7 +7940,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ZMO0820</t>
+          <t>ZMO1531</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -7974,7 +7974,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ZMO1531</t>
+          <t>ZMO1532</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -8008,7 +8008,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ZMO1532</t>
+          <t>ZMO0820</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -8348,7 +8348,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ZMO1421</t>
+          <t>ZMO1420</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -8382,7 +8382,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ZMO1420</t>
+          <t>ZMO1421</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -8688,7 +8688,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ZMO1278</t>
+          <t>ZMO1899</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -8722,7 +8722,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ZMO1899</t>
+          <t>ZMO1278</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -8892,7 +8892,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ZMO1278</t>
+          <t>ZMO1899</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -8926,7 +8926,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ZMO1899</t>
+          <t>ZMO1278</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -9028,7 +9028,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ZMO1868</t>
+          <t>ZMO0735</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -9096,7 +9096,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ZMO0735</t>
+          <t>ZMO1868</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -9130,7 +9130,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ZMO0583</t>
+          <t>ZMO0599</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -9164,7 +9164,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ZMO0599</t>
+          <t>ZMO0583</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -9266,7 +9266,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ZMO1050</t>
+          <t>ZMO1049</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -9334,7 +9334,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ZMO1049</t>
+          <t>ZMO1050</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -9402,7 +9402,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ZMO0443</t>
+          <t>ZMO0573</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -9538,7 +9538,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ZMO0573</t>
+          <t>ZMO0443</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">

</xml_diff>